<commit_message>
Further changes before starting
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
+++ b/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_FU_SHORT\Forms\MADTRIAL_FU_SHORT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08428C3-A3B6-42C4-BC9A-7A7840D0D4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536C8B00-5D99-4891-B6C8-3CB0D34DD8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="365">
   <si>
     <t>setting_name</t>
   </si>
@@ -1149,6 +1149,9 @@
   </si>
   <si>
     <t>MADtrial - Seguimento Chamada EA</t>
+  </si>
+  <si>
+    <t>SARVAC</t>
   </si>
 </sst>
 </file>
@@ -6056,7 +6059,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.7265625" customWidth="1"/>
@@ -6409,7 +6412,7 @@
         <v>46</v>
       </c>
       <c r="C27" s="8" t="b">
-        <f t="shared" ref="C27:C67" si="3">FALSE()</f>
+        <f t="shared" ref="C27:C68" si="3">FALSE()</f>
         <v>0</v>
       </c>
       <c r="D27" s="8"/>
@@ -6583,25 +6586,24 @@
       </c>
       <c r="D40" s="8"/>
     </row>
-    <row r="41" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="8" t="s">
-        <v>170</v>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>364</v>
       </c>
       <c r="B41" t="s">
-        <v>169</v>
-      </c>
-      <c r="C41" s="1" t="b">
-        <f t="shared" si="3"/>
+        <v>60</v>
+      </c>
+      <c r="C41" t="b">
         <v>0</v>
       </c>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B42" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="C42" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6611,10 +6613,10 @@
     </row>
     <row r="43" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B43" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C43" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6624,10 +6626,10 @@
     </row>
     <row r="44" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B44" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C44" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6637,10 +6639,10 @@
     </row>
     <row r="45" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B45" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C45" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6650,10 +6652,10 @@
     </row>
     <row r="46" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B46" t="s">
-        <v>182</v>
+        <v>60</v>
       </c>
       <c r="C46" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6663,22 +6665,23 @@
     </row>
     <row r="47" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B47" t="s">
-        <v>60</v>
+        <v>182</v>
       </c>
       <c r="C47" s="1" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B48" t="s">
-        <v>182</v>
+        <v>60</v>
       </c>
       <c r="C48" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6687,10 +6690,10 @@
     </row>
     <row r="49" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B49" t="s">
-        <v>60</v>
+        <v>182</v>
       </c>
       <c r="C49" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6699,10 +6702,10 @@
     </row>
     <row r="50" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
+      </c>
+      <c r="B50" t="s">
+        <v>60</v>
       </c>
       <c r="C50" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6711,10 +6714,10 @@
     </row>
     <row r="51" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>60</v>
+        <v>182</v>
       </c>
       <c r="C51" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6723,10 +6726,10 @@
     </row>
     <row r="52" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C52" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6735,10 +6738,10 @@
     </row>
     <row r="53" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C53" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6747,10 +6750,10 @@
     </row>
     <row r="54" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C54" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6759,10 +6762,10 @@
     </row>
     <row r="55" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C55" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6771,10 +6774,10 @@
     </row>
     <row r="56" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C56" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6783,10 +6786,10 @@
     </row>
     <row r="57" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C57" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6795,10 +6798,10 @@
     </row>
     <row r="58" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="8" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>202</v>
+        <v>60</v>
       </c>
       <c r="C58" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6807,10 +6810,10 @@
     </row>
     <row r="59" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="8" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>151</v>
+        <v>202</v>
       </c>
       <c r="C59" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6818,11 +6821,11 @@
       </c>
     </row>
     <row r="60" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="1" t="s">
-        <v>207</v>
+      <c r="A60" s="8" t="s">
+        <v>206</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>60</v>
+        <v>151</v>
       </c>
       <c r="C60" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6830,11 +6833,11 @@
       </c>
     </row>
     <row r="61" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="8" t="s">
-        <v>211</v>
+      <c r="A61" s="1" t="s">
+        <v>207</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C61" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6843,10 +6846,10 @@
     </row>
     <row r="62" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>202</v>
+        <v>151</v>
       </c>
       <c r="C62" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6855,10 +6858,10 @@
     </row>
     <row r="63" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A63" s="8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>60</v>
+        <v>202</v>
       </c>
       <c r="C63" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6867,7 +6870,7 @@
     </row>
     <row r="64" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>60</v>
@@ -6879,10 +6882,10 @@
     </row>
     <row r="65" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A65" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C65" s="1" t="b">
         <f t="shared" si="3"/>
@@ -6890,23 +6893,23 @@
       </c>
     </row>
     <row r="66" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="15" t="s">
-        <v>222</v>
-      </c>
-      <c r="B66" t="s">
+      <c r="A66" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C66" s="8" t="b">
+      <c r="C66" s="1" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A67" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="B67" s="8" t="s">
-        <v>202</v>
+        <v>222</v>
+      </c>
+      <c r="B67" t="s">
+        <v>151</v>
       </c>
       <c r="C67" s="8" t="b">
         <f t="shared" si="3"/>
@@ -6914,29 +6917,30 @@
       </c>
     </row>
     <row r="68" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="8"/>
-      <c r="B68" s="8"/>
-      <c r="C68" s="8"/>
+      <c r="A68" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C68" s="8" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="69" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>145</v>
-      </c>
-      <c r="B70" t="s">
-        <v>46</v>
-      </c>
-      <c r="C70" t="b">
-        <v>0</v>
-      </c>
+    <row r="70" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="8"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>347</v>
+        <v>145</v>
       </c>
       <c r="B71" t="s">
         <v>46</v>
@@ -6947,7 +6951,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B72" t="s">
         <v>46</v>
@@ -6958,12 +6962,23 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
+        <v>348</v>
+      </c>
+      <c r="B73" t="s">
+        <v>46</v>
+      </c>
+      <c r="C73" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>134</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>36</v>
       </c>
-      <c r="C73" t="b">
+      <c r="C74" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Further changes before start
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
+++ b/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_FU_SHORT\Forms\MADTRIAL_FU_SHORT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536C8B00-5D99-4891-B6C8-3CB0D34DD8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB6E67B-3A40-4DD6-9638-B73F745A7B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -1590,7 +1590,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P274"/>
+  <dimension ref="A1:P286"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.453125" customWidth="1"/>
@@ -4134,13 +4134,24 @@
         <v>128</v>
       </c>
     </row>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B273" t="s">
+    <row r="284" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="D284" t="s">
+        <v>36</v>
+      </c>
+      <c r="F284" t="s">
+        <v>134</v>
+      </c>
+      <c r="I284" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="285" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B285" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B274" t="s">
+    <row r="286" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B286" t="s">
         <v>50</v>
       </c>
     </row>
@@ -4226,17 +4237,6 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="D3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" t="s">
-        <v>134</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>135</v>
-      </c>
-    </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D4" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
Fitering for 9 months FU*
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
+++ b/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_FU_SHORT\Forms\MADTRIAL_FU_SHORT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB6E67B-3A40-4DD6-9638-B73F745A7B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F1A871-AB1C-4704-B84A-99899585D74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Corrections to index and question phrasing for short FU
</commit_message>
<xml_diff>
--- a/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
+++ b/app/config/tables/MADTRIAL_FU_SHORT/Forms/MADTRIAL_FU_SHORT/MADTRIAL_FU_SHORT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MADtrials2\MADtrial\app\config\tables\MADTRIAL_FU_SHORT\Forms\MADTRIAL_FU_SHORT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afisker\Documents\tablet\MAD_2_2\MADtrial\app\config\tables\MADTRIAL_FU_SHORT\Forms\MADTRIAL_FU_SHORT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8F1A871-AB1C-4704-B84A-99899585D74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F322BB-2D2B-4EEF-9B93-79F2FE61BF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -1106,42 +1106,12 @@
     <t>DATINC</t>
   </si>
   <si>
-    <t>A criança teve diarréia durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança vomitou  durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança teve tosse  durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança está com constipação  durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança perdeu o seu apetite durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança chorou mais do que o habitual durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança teve febre  durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança teve convulsões (desmaio) durante ultimo semana?</t>
-  </si>
-  <si>
-    <t>A criança teve outras sintomas durante ultimo semana?</t>
-  </si>
-  <si>
     <t>Augusto da Costa</t>
   </si>
   <si>
     <t>Josemira</t>
   </si>
   <si>
-    <t>A criança recebeu medicamentos durante ultimo semana?</t>
-  </si>
-  <si>
     <t>Inclusão/Último seguimento por telefone: &lt;b&gt;{{calculates.displayLASTFUSUC}}&lt;/b&gt;</t>
   </si>
   <si>
@@ -1152,6 +1122,36 @@
   </si>
   <si>
     <t>SARVAC</t>
+  </si>
+  <si>
+    <t>A criança teve convulsões (ataque) durante ultimo semana?</t>
+  </si>
+  <si>
+    <t>A criança chorou mais do que o habitual durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança teve febre  durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança teve outras sintomas durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança perdeu o seu apetite durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança está com constipação  durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança teve tosse  durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança vomitou  durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança teve diarréia durante ultimo semana? (Se sim - este e novo sintoma, ou aquele com que ele(a) saiu do HNSM com?)</t>
+  </si>
+  <si>
+    <t>A criança recebeu medicamentos durante a ultima semana? (Se sim - são novos medicamentos, ou aqueles receitados no HNSM?)</t>
   </si>
 </sst>
 </file>
@@ -1546,10 +1546,10 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="D5" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -4420,7 +4420,7 @@
         <v>168</v>
       </c>
       <c r="H24" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.35">
@@ -4437,7 +4437,7 @@
         <v>171</v>
       </c>
       <c r="H25" t="s">
-        <v>349</v>
+        <v>363</v>
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.35">
@@ -4461,7 +4461,7 @@
         <v>168</v>
       </c>
       <c r="H33" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.35">
@@ -4478,7 +4478,7 @@
         <v>178</v>
       </c>
       <c r="H34" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.35">
@@ -4502,7 +4502,7 @@
         <v>168</v>
       </c>
       <c r="H40" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.35">
@@ -4519,7 +4519,7 @@
         <v>181</v>
       </c>
       <c r="H41" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="43" spans="2:11" x14ac:dyDescent="0.35">
@@ -4543,7 +4543,7 @@
         <v>168</v>
       </c>
       <c r="H47" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.35">
@@ -4560,7 +4560,7 @@
         <v>185</v>
       </c>
       <c r="H48" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.35">
@@ -4584,7 +4584,7 @@
         <v>168</v>
       </c>
       <c r="H54" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.35">
@@ -4601,7 +4601,7 @@
         <v>188</v>
       </c>
       <c r="H55" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.35">
@@ -4625,7 +4625,7 @@
         <v>168</v>
       </c>
       <c r="H61" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.35">
@@ -4642,7 +4642,7 @@
         <v>191</v>
       </c>
       <c r="H62" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.35">
@@ -4666,7 +4666,7 @@
         <v>168</v>
       </c>
       <c r="H68" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.35">
@@ -4683,7 +4683,7 @@
         <v>194</v>
       </c>
       <c r="H69" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.35">
@@ -4707,7 +4707,7 @@
         <v>168</v>
       </c>
       <c r="H75" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.35">
@@ -4724,7 +4724,7 @@
         <v>197</v>
       </c>
       <c r="H76" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.35">
@@ -4748,7 +4748,7 @@
         <v>168</v>
       </c>
       <c r="H82" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="83" spans="2:11" x14ac:dyDescent="0.35">
@@ -4765,7 +4765,7 @@
         <v>200</v>
       </c>
       <c r="H83" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.35">
@@ -4816,7 +4816,7 @@
         <v>168</v>
       </c>
       <c r="H90" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="91" spans="2:11" x14ac:dyDescent="0.35">
@@ -4901,7 +4901,7 @@
         <v>168</v>
       </c>
       <c r="H99" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.35">
@@ -4918,7 +4918,7 @@
         <v>218</v>
       </c>
       <c r="H100" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
     <row r="101" spans="2:11" x14ac:dyDescent="0.35">
@@ -5176,10 +5176,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="D8" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="G8" s="8"/>
     </row>
@@ -5192,10 +5192,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="D9" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="G9" s="8"/>
     </row>
@@ -6588,7 +6588,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="B41" t="s">
         <v>60</v>

</xml_diff>